<commit_message>
feat: add itinerary screen and home travel card
</commit_message>
<xml_diff>
--- a/assets/region_codes.xlsx
+++ b/assets/region_codes.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\1.업무공통\TourAPI\5.신규_OpenAPI_빅데이터\OpenAPI매뉴얼작업_240604\TourAPI_Guide_(기초지자체_중심관광지정보)v4.0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\SNOB\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C67998A-9111-49CF-81B8-236F02140736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13110"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시도,시군구코드" sheetId="1" r:id="rId1"/>
@@ -530,9 +531,6 @@
     <t>부안군</t>
   </si>
   <si>
-    <t>전라남도</t>
-  </si>
-  <si>
     <t>목포시</t>
   </si>
   <si>
@@ -777,13 +775,17 @@
   </si>
   <si>
     <t>sigunguNm</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>전남광주통합특별시</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -853,7 +855,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -864,12 +866,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1151,31 +1147,31 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D253"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="7.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.08203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.25" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" s="2">
         <v>11</v>
       </c>
@@ -1189,7 +1185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" s="2">
         <v>11</v>
       </c>
@@ -1203,7 +1199,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" s="2">
         <v>11</v>
       </c>
@@ -1217,7 +1213,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" s="2">
         <v>11</v>
       </c>
@@ -1231,7 +1227,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" s="2">
         <v>11</v>
       </c>
@@ -1245,7 +1241,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" s="2">
         <v>11</v>
       </c>
@@ -1259,7 +1255,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" s="2">
         <v>11</v>
       </c>
@@ -1273,7 +1269,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" s="2">
         <v>11</v>
       </c>
@@ -1287,7 +1283,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" s="2">
         <v>11</v>
       </c>
@@ -1301,7 +1297,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" s="2">
         <v>11</v>
       </c>
@@ -1315,7 +1311,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1329,7 +1325,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" s="2">
         <v>11</v>
       </c>
@@ -1343,7 +1339,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" s="2">
         <v>11</v>
       </c>
@@ -1357,7 +1353,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" s="2">
         <v>11</v>
       </c>
@@ -1371,7 +1367,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" s="2">
         <v>11</v>
       </c>
@@ -1385,7 +1381,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A17" s="2">
         <v>11</v>
       </c>
@@ -1399,7 +1395,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A18" s="2">
         <v>11</v>
       </c>
@@ -1413,7 +1409,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A19" s="2">
         <v>11</v>
       </c>
@@ -1427,7 +1423,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A20" s="2">
         <v>11</v>
       </c>
@@ -1441,7 +1437,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" s="2">
         <v>11</v>
       </c>
@@ -1455,7 +1451,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A22" s="2">
         <v>11</v>
       </c>
@@ -1469,7 +1465,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" s="2">
         <v>11</v>
       </c>
@@ -1483,7 +1479,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" s="2">
         <v>11</v>
       </c>
@@ -1497,7 +1493,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A25" s="2">
         <v>11</v>
       </c>
@@ -1511,7 +1507,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A26" s="2">
         <v>11</v>
       </c>
@@ -1525,7 +1521,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1539,7 +1535,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A28" s="2">
         <v>26</v>
       </c>
@@ -1553,7 +1549,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A29" s="2">
         <v>26</v>
       </c>
@@ -1567,7 +1563,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A30" s="2">
         <v>26</v>
       </c>
@@ -1581,7 +1577,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A31" s="2">
         <v>26</v>
       </c>
@@ -1595,7 +1591,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A32" s="2">
         <v>26</v>
       </c>
@@ -1609,7 +1605,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A33" s="2">
         <v>26</v>
       </c>
@@ -1623,7 +1619,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A34" s="2">
         <v>26</v>
       </c>
@@ -1637,7 +1633,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A35" s="2">
         <v>26</v>
       </c>
@@ -1651,7 +1647,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A36" s="2">
         <v>26</v>
       </c>
@@ -1665,7 +1661,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A37" s="2">
         <v>26</v>
       </c>
@@ -1679,7 +1675,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A38" s="2">
         <v>26</v>
       </c>
@@ -1693,7 +1689,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A39" s="2">
         <v>26</v>
       </c>
@@ -1707,7 +1703,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A40" s="2">
         <v>26</v>
       </c>
@@ -1721,7 +1717,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A41" s="2">
         <v>26</v>
       </c>
@@ -1735,7 +1731,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A42" s="2">
         <v>26</v>
       </c>
@@ -1749,7 +1745,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A43" s="2">
         <v>27</v>
       </c>
@@ -1763,7 +1759,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A44" s="2">
         <v>27</v>
       </c>
@@ -1777,7 +1773,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A45" s="2">
         <v>27</v>
       </c>
@@ -1791,7 +1787,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A46" s="2">
         <v>27</v>
       </c>
@@ -1805,7 +1801,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A47" s="2">
         <v>27</v>
       </c>
@@ -1819,7 +1815,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A48" s="2">
         <v>27</v>
       </c>
@@ -1833,7 +1829,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A49" s="2">
         <v>27</v>
       </c>
@@ -1847,7 +1843,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A50" s="2">
         <v>27</v>
       </c>
@@ -1861,7 +1857,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A51" s="2">
         <v>27</v>
       </c>
@@ -1872,10 +1868,10 @@
         <v>27720</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A52" s="2">
         <v>28</v>
       </c>
@@ -1889,7 +1885,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A53" s="2">
         <v>28</v>
       </c>
@@ -1903,7 +1899,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A54" s="2">
         <v>28</v>
       </c>
@@ -1917,7 +1913,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A55" s="2">
         <v>28</v>
       </c>
@@ -1931,7 +1927,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A56" s="2">
         <v>28</v>
       </c>
@@ -1945,7 +1941,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A57" s="2">
         <v>28</v>
       </c>
@@ -1959,7 +1955,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A58" s="2">
         <v>28</v>
       </c>
@@ -1973,7 +1969,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A59" s="2">
         <v>28</v>
       </c>
@@ -1987,7 +1983,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A60" s="2">
         <v>28</v>
       </c>
@@ -2001,7 +1997,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A61" s="2">
         <v>28</v>
       </c>
@@ -2015,7 +2011,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A62" s="2">
         <v>29</v>
       </c>
@@ -2029,7 +2025,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A63" s="2">
         <v>29</v>
       </c>
@@ -2043,7 +2039,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A64" s="2">
         <v>29</v>
       </c>
@@ -2057,7 +2053,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A65" s="2">
         <v>29</v>
       </c>
@@ -2071,7 +2067,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A66" s="2">
         <v>29</v>
       </c>
@@ -2085,7 +2081,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A67" s="2">
         <v>30</v>
       </c>
@@ -2099,7 +2095,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A68" s="2">
         <v>30</v>
       </c>
@@ -2113,7 +2109,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A69" s="2">
         <v>30</v>
       </c>
@@ -2127,7 +2123,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A70" s="2">
         <v>30</v>
       </c>
@@ -2141,7 +2137,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A71" s="2">
         <v>30</v>
       </c>
@@ -2155,7 +2151,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A72" s="2">
         <v>31</v>
       </c>
@@ -2169,7 +2165,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A73" s="2">
         <v>31</v>
       </c>
@@ -2183,7 +2179,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A74" s="2">
         <v>31</v>
       </c>
@@ -2197,7 +2193,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A75" s="2">
         <v>31</v>
       </c>
@@ -2211,7 +2207,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A76" s="2">
         <v>31</v>
       </c>
@@ -2225,7 +2221,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A77" s="2">
         <v>36</v>
       </c>
@@ -2239,7 +2235,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A78" s="2">
         <v>41</v>
       </c>
@@ -2253,7 +2249,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A79" s="2">
         <v>41</v>
       </c>
@@ -2267,7 +2263,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A80" s="2">
         <v>41</v>
       </c>
@@ -2281,7 +2277,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A81" s="2">
         <v>41</v>
       </c>
@@ -2295,7 +2291,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A82" s="2">
         <v>41</v>
       </c>
@@ -2309,7 +2305,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A83" s="2">
         <v>41</v>
       </c>
@@ -2323,7 +2319,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A84" s="2">
         <v>41</v>
       </c>
@@ -2337,7 +2333,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A85" s="2">
         <v>41</v>
       </c>
@@ -2351,7 +2347,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A86" s="2">
         <v>41</v>
       </c>
@@ -2365,7 +2361,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A87" s="2">
         <v>41</v>
       </c>
@@ -2379,49 +2375,49 @@
         <v>71</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A88" s="4">
-        <v>41</v>
-      </c>
-      <c r="B88" s="5" t="s">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A88" s="2">
+        <v>41</v>
+      </c>
+      <c r="B88" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C88" s="4">
+      <c r="C88" s="2">
         <v>41192</v>
       </c>
-      <c r="D88" s="5" t="s">
+      <c r="D88" s="3" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A89" s="2">
+        <v>41</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C89" s="2">
+        <v>41194</v>
+      </c>
+      <c r="D89" s="3" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A89" s="4">
-        <v>41</v>
-      </c>
-      <c r="B89" s="5" t="s">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A90" s="2">
+        <v>41</v>
+      </c>
+      <c r="B90" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C89" s="4">
-        <v>41194</v>
-      </c>
-      <c r="D89" s="5" t="s">
+      <c r="C90" s="2">
+        <v>41196</v>
+      </c>
+      <c r="D90" s="3" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A90" s="4">
-        <v>41</v>
-      </c>
-      <c r="B90" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="C90" s="4">
-        <v>41196</v>
-      </c>
-      <c r="D90" s="5" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A91" s="2">
         <v>41</v>
       </c>
@@ -2435,7 +2431,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A92" s="2">
         <v>41</v>
       </c>
@@ -2449,7 +2445,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A93" s="2">
         <v>41</v>
       </c>
@@ -2463,7 +2459,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A94" s="2">
         <v>41</v>
       </c>
@@ -2477,7 +2473,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A95" s="2">
         <v>41</v>
       </c>
@@ -2491,7 +2487,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A96" s="2">
         <v>41</v>
       </c>
@@ -2505,7 +2501,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A97" s="2">
         <v>41</v>
       </c>
@@ -2519,7 +2515,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A98" s="2">
         <v>41</v>
       </c>
@@ -2533,7 +2529,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A99" s="2">
         <v>41</v>
       </c>
@@ -2547,7 +2543,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A100" s="2">
         <v>41</v>
       </c>
@@ -2561,7 +2557,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A101" s="2">
         <v>41</v>
       </c>
@@ -2575,7 +2571,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A102" s="2">
         <v>41</v>
       </c>
@@ -2589,7 +2585,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A103" s="2">
         <v>41</v>
       </c>
@@ -2603,7 +2599,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A104" s="2">
         <v>41</v>
       </c>
@@ -2617,7 +2613,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A105" s="2">
         <v>41</v>
       </c>
@@ -2631,7 +2627,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A106" s="2">
         <v>41</v>
       </c>
@@ -2645,7 +2641,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A107" s="2">
         <v>41</v>
       </c>
@@ -2659,7 +2655,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A108" s="2">
         <v>41</v>
       </c>
@@ -2673,7 +2669,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A109" s="2">
         <v>41</v>
       </c>
@@ -2687,7 +2683,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A110" s="2">
         <v>41</v>
       </c>
@@ -2701,7 +2697,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A111" s="2">
         <v>41</v>
       </c>
@@ -2715,7 +2711,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A112" s="2">
         <v>41</v>
       </c>
@@ -2729,7 +2725,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A113" s="2">
         <v>41</v>
       </c>
@@ -2743,7 +2739,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A114" s="2">
         <v>41</v>
       </c>
@@ -2757,7 +2753,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A115" s="2">
         <v>41</v>
       </c>
@@ -2771,7 +2767,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A116" s="2">
         <v>41</v>
       </c>
@@ -2785,7 +2781,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A117" s="2">
         <v>41</v>
       </c>
@@ -2799,7 +2795,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A118" s="2">
         <v>41</v>
       </c>
@@ -2813,7 +2809,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A119" s="2">
         <v>41</v>
       </c>
@@ -2827,7 +2823,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A120" s="2">
         <v>41</v>
       </c>
@@ -2841,7 +2837,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A121" s="2">
         <v>41</v>
       </c>
@@ -2855,7 +2851,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A122" s="2">
         <v>43</v>
       </c>
@@ -2869,7 +2865,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A123" s="2">
         <v>43</v>
       </c>
@@ -2883,7 +2879,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A124" s="2">
         <v>43</v>
       </c>
@@ -2897,7 +2893,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A125" s="2">
         <v>43</v>
       </c>
@@ -2911,7 +2907,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A126" s="2">
         <v>43</v>
       </c>
@@ -2925,7 +2921,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A127" s="2">
         <v>43</v>
       </c>
@@ -2939,7 +2935,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A128" s="2">
         <v>43</v>
       </c>
@@ -2953,7 +2949,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A129" s="2">
         <v>43</v>
       </c>
@@ -2967,7 +2963,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A130" s="2">
         <v>43</v>
       </c>
@@ -2981,7 +2977,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A131" s="2">
         <v>43</v>
       </c>
@@ -2995,7 +2991,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A132" s="2">
         <v>43</v>
       </c>
@@ -3009,7 +3005,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A133" s="2">
         <v>43</v>
       </c>
@@ -3023,7 +3019,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A134" s="2">
         <v>43</v>
       </c>
@@ -3037,7 +3033,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A135" s="2">
         <v>43</v>
       </c>
@@ -3051,7 +3047,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A136" s="2">
         <v>44</v>
       </c>
@@ -3065,7 +3061,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A137" s="2">
         <v>44</v>
       </c>
@@ -3079,7 +3075,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A138" s="2">
         <v>44</v>
       </c>
@@ -3093,7 +3089,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A139" s="2">
         <v>44</v>
       </c>
@@ -3107,7 +3103,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A140" s="2">
         <v>44</v>
       </c>
@@ -3121,7 +3117,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A141" s="2">
         <v>44</v>
       </c>
@@ -3135,7 +3131,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A142" s="2">
         <v>44</v>
       </c>
@@ -3149,7 +3145,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A143" s="2">
         <v>44</v>
       </c>
@@ -3163,7 +3159,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A144" s="2">
         <v>44</v>
       </c>
@@ -3177,7 +3173,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A145" s="2">
         <v>44</v>
       </c>
@@ -3191,7 +3187,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A146" s="2">
         <v>44</v>
       </c>
@@ -3205,7 +3201,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A147" s="2">
         <v>44</v>
       </c>
@@ -3219,7 +3215,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A148" s="2">
         <v>44</v>
       </c>
@@ -3233,7 +3229,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A149" s="2">
         <v>44</v>
       </c>
@@ -3247,7 +3243,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A150" s="2">
         <v>44</v>
       </c>
@@ -3261,7 +3257,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A151" s="2">
         <v>44</v>
       </c>
@@ -3275,852 +3271,852 @@
         <v>152</v>
       </c>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A152" s="2">
         <v>46</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C152" s="2">
         <v>46110</v>
       </c>
       <c r="D152" s="3" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A153" s="2">
         <v>46</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C153" s="2">
         <v>46130</v>
       </c>
       <c r="D153" s="3" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A154" s="2">
         <v>46</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C154" s="2">
         <v>46150</v>
       </c>
       <c r="D154" s="3" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A155" s="2">
         <v>46</v>
       </c>
       <c r="B155" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C155" s="2">
         <v>46170</v>
       </c>
       <c r="D155" s="3" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A156" s="2">
         <v>46</v>
       </c>
       <c r="B156" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C156" s="2">
         <v>46230</v>
       </c>
       <c r="D156" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A157" s="2">
         <v>46</v>
       </c>
       <c r="B157" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C157" s="2">
         <v>46710</v>
       </c>
       <c r="D157" s="3" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A158" s="2">
         <v>46</v>
       </c>
       <c r="B158" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C158" s="2">
         <v>46720</v>
       </c>
       <c r="D158" s="3" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A159" s="2">
         <v>46</v>
       </c>
       <c r="B159" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C159" s="2">
         <v>46730</v>
       </c>
       <c r="D159" s="3" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A160" s="2">
         <v>46</v>
       </c>
       <c r="B160" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C160" s="2">
         <v>46770</v>
       </c>
       <c r="D160" s="3" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A161" s="2">
         <v>46</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C161" s="2">
         <v>46780</v>
       </c>
       <c r="D161" s="3" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A162" s="2">
         <v>46</v>
       </c>
       <c r="B162" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C162" s="2">
         <v>46790</v>
       </c>
       <c r="D162" s="3" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A163" s="2">
         <v>46</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C163" s="2">
         <v>46800</v>
       </c>
       <c r="D163" s="3" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.3">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A164" s="2">
         <v>46</v>
       </c>
       <c r="B164" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C164" s="2">
         <v>46810</v>
       </c>
       <c r="D164" s="3" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.3">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A165" s="2">
         <v>46</v>
       </c>
       <c r="B165" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C165" s="2">
         <v>46820</v>
       </c>
       <c r="D165" s="3" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.3">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A166" s="2">
         <v>46</v>
       </c>
       <c r="B166" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C166" s="2">
         <v>46830</v>
       </c>
       <c r="D166" s="3" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.3">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A167" s="2">
         <v>46</v>
       </c>
       <c r="B167" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C167" s="2">
         <v>46840</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.3">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A168" s="2">
         <v>46</v>
       </c>
       <c r="B168" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C168" s="2">
         <v>46860</v>
       </c>
       <c r="D168" s="3" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.3">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A169" s="2">
         <v>46</v>
       </c>
       <c r="B169" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C169" s="2">
         <v>46870</v>
       </c>
       <c r="D169" s="3" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.3">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A170" s="2">
         <v>46</v>
       </c>
       <c r="B170" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C170" s="2">
         <v>46880</v>
       </c>
       <c r="D170" s="3" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.3">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A171" s="2">
         <v>46</v>
       </c>
       <c r="B171" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C171" s="2">
         <v>46890</v>
       </c>
       <c r="D171" s="3" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.3">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A172" s="2">
         <v>46</v>
       </c>
       <c r="B172" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C172" s="2">
         <v>46900</v>
       </c>
       <c r="D172" s="3" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.3">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A173" s="2">
         <v>46</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>168</v>
+        <v>249</v>
       </c>
       <c r="C173" s="2">
         <v>46910</v>
       </c>
       <c r="D173" s="3" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.3">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A174" s="2">
         <v>47</v>
       </c>
       <c r="B174" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C174" s="2">
         <v>47111</v>
       </c>
       <c r="D174" s="3" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.3">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A175" s="2">
         <v>47</v>
       </c>
       <c r="B175" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C175" s="2">
         <v>47113</v>
       </c>
       <c r="D175" s="3" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.3">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A176" s="2">
         <v>47</v>
       </c>
       <c r="B176" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C176" s="2">
         <v>47130</v>
       </c>
       <c r="D176" s="3" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.3">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A177" s="2">
         <v>47</v>
       </c>
       <c r="B177" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C177" s="2">
         <v>47150</v>
       </c>
       <c r="D177" s="3" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.3">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A178" s="2">
         <v>47</v>
       </c>
       <c r="B178" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C178" s="2">
         <v>47170</v>
       </c>
       <c r="D178" s="3" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.3">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A179" s="2">
         <v>47</v>
       </c>
       <c r="B179" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C179" s="2">
         <v>47190</v>
       </c>
       <c r="D179" s="3" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.3">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A180" s="2">
         <v>47</v>
       </c>
       <c r="B180" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C180" s="2">
         <v>47210</v>
       </c>
       <c r="D180" s="3" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.3">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A181" s="2">
         <v>47</v>
       </c>
       <c r="B181" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C181" s="2">
         <v>47230</v>
       </c>
       <c r="D181" s="3" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.3">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A182" s="2">
         <v>47</v>
       </c>
       <c r="B182" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C182" s="2">
         <v>47250</v>
       </c>
       <c r="D182" s="3" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.3">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A183" s="2">
         <v>47</v>
       </c>
       <c r="B183" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C183" s="2">
         <v>47280</v>
       </c>
       <c r="D183" s="3" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.3">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A184" s="2">
         <v>47</v>
       </c>
       <c r="B184" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C184" s="2">
         <v>47290</v>
       </c>
       <c r="D184" s="3" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.3">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A185" s="2">
         <v>47</v>
       </c>
       <c r="B185" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C185" s="2">
         <v>47730</v>
       </c>
       <c r="D185" s="3" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.3">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A186" s="2">
         <v>47</v>
       </c>
       <c r="B186" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C186" s="2">
         <v>47750</v>
       </c>
       <c r="D186" s="3" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.3">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A187" s="2">
         <v>47</v>
       </c>
       <c r="B187" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C187" s="2">
         <v>47760</v>
       </c>
       <c r="D187" s="3" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.3">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A188" s="2">
         <v>47</v>
       </c>
       <c r="B188" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C188" s="2">
         <v>47770</v>
       </c>
       <c r="D188" s="3" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.3">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A189" s="2">
         <v>47</v>
       </c>
       <c r="B189" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C189" s="2">
         <v>47820</v>
       </c>
       <c r="D189" s="3" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.3">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A190" s="2">
         <v>47</v>
       </c>
       <c r="B190" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C190" s="2">
         <v>47830</v>
       </c>
       <c r="D190" s="3" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.3">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A191" s="2">
         <v>47</v>
       </c>
       <c r="B191" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C191" s="2">
         <v>47840</v>
       </c>
       <c r="D191" s="3" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.3">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A192" s="2">
         <v>47</v>
       </c>
       <c r="B192" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C192" s="2">
         <v>47850</v>
       </c>
       <c r="D192" s="3" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.3">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A193" s="2">
         <v>47</v>
       </c>
       <c r="B193" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C193" s="2">
         <v>47900</v>
       </c>
       <c r="D193" s="3" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.3">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A194" s="2">
         <v>47</v>
       </c>
       <c r="B194" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C194" s="2">
         <v>47920</v>
       </c>
       <c r="D194" s="3" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.3">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A195" s="2">
         <v>47</v>
       </c>
       <c r="B195" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C195" s="2">
         <v>47930</v>
       </c>
       <c r="D195" s="3" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.3">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A196" s="2">
         <v>47</v>
       </c>
       <c r="B196" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C196" s="2">
         <v>47940</v>
       </c>
       <c r="D196" s="3" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.3">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A197" s="2">
         <v>48</v>
       </c>
       <c r="B197" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C197" s="2">
         <v>48121</v>
       </c>
       <c r="D197" s="3" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.3">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A198" s="2">
         <v>48</v>
       </c>
       <c r="B198" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C198" s="2">
         <v>48123</v>
       </c>
       <c r="D198" s="3" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.3">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="199" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A199" s="2">
         <v>48</v>
       </c>
       <c r="B199" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C199" s="2">
         <v>48125</v>
       </c>
       <c r="D199" s="3" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.3">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="200" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A200" s="2">
         <v>48</v>
       </c>
       <c r="B200" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C200" s="2">
         <v>48127</v>
       </c>
       <c r="D200" s="3" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.3">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="201" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A201" s="2">
         <v>48</v>
       </c>
       <c r="B201" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C201" s="2">
         <v>48129</v>
       </c>
       <c r="D201" s="3" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.3">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="202" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A202" s="2">
         <v>48</v>
       </c>
       <c r="B202" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C202" s="2">
         <v>48170</v>
       </c>
       <c r="D202" s="3" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.3">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A203" s="2">
         <v>48</v>
       </c>
       <c r="B203" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C203" s="2">
         <v>48220</v>
       </c>
       <c r="D203" s="3" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.3">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A204" s="2">
         <v>48</v>
       </c>
       <c r="B204" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C204" s="2">
         <v>48240</v>
       </c>
       <c r="D204" s="3" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.3">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="205" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A205" s="2">
         <v>48</v>
       </c>
       <c r="B205" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C205" s="2">
         <v>48250</v>
       </c>
       <c r="D205" s="3" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.3">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="206" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A206" s="2">
         <v>48</v>
       </c>
       <c r="B206" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C206" s="2">
         <v>48270</v>
       </c>
       <c r="D206" s="3" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.3">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="207" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A207" s="2">
         <v>48</v>
       </c>
       <c r="B207" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C207" s="2">
         <v>48310</v>
       </c>
       <c r="D207" s="3" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.3">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="208" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A208" s="2">
         <v>48</v>
       </c>
       <c r="B208" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C208" s="2">
         <v>48330</v>
       </c>
       <c r="D208" s="3" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.3">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="209" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A209" s="2">
         <v>48</v>
       </c>
       <c r="B209" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C209" s="2">
         <v>48720</v>
       </c>
       <c r="D209" s="3" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.3">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="210" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A210" s="2">
         <v>48</v>
       </c>
       <c r="B210" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C210" s="2">
         <v>48730</v>
       </c>
       <c r="D210" s="3" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.3">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="211" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A211" s="2">
         <v>48</v>
       </c>
       <c r="B211" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C211" s="2">
         <v>48740</v>
       </c>
       <c r="D211" s="3" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.3">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="212" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A212" s="2">
         <v>48</v>
       </c>
       <c r="B212" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C212" s="2">
         <v>48820</v>
@@ -4129,124 +4125,124 @@
         <v>119</v>
       </c>
     </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A213" s="2">
         <v>48</v>
       </c>
       <c r="B213" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C213" s="2">
         <v>48840</v>
       </c>
       <c r="D213" s="3" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.3">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="214" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A214" s="2">
         <v>48</v>
       </c>
       <c r="B214" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C214" s="2">
         <v>48850</v>
       </c>
       <c r="D214" s="3" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.3">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="215" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A215" s="2">
         <v>48</v>
       </c>
       <c r="B215" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C215" s="2">
         <v>48860</v>
       </c>
       <c r="D215" s="3" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="216" spans="1:4" x14ac:dyDescent="0.3">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="216" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A216" s="2">
         <v>48</v>
       </c>
       <c r="B216" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C216" s="2">
         <v>48870</v>
       </c>
       <c r="D216" s="3" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.3">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="217" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A217" s="2">
         <v>48</v>
       </c>
       <c r="B217" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C217" s="2">
         <v>48880</v>
       </c>
       <c r="D217" s="3" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.3">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="218" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A218" s="2">
         <v>48</v>
       </c>
       <c r="B218" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C218" s="2">
         <v>48890</v>
       </c>
       <c r="D218" s="3" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="219" spans="1:4" x14ac:dyDescent="0.3">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="219" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A219" s="2">
         <v>50</v>
       </c>
       <c r="B219" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C219" s="2">
         <v>50110</v>
       </c>
       <c r="D219" s="3" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="220" spans="1:4" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="220" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A220" s="2">
         <v>50</v>
       </c>
       <c r="B220" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C220" s="2">
         <v>50130</v>
       </c>
       <c r="D220" s="3" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.3">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="221" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A221" s="2">
         <v>51</v>
       </c>
       <c r="B221" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C221" s="2">
         <v>51110</v>
@@ -4255,12 +4251,12 @@
         <v>103</v>
       </c>
     </row>
-    <row r="222" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A222" s="2">
         <v>51</v>
       </c>
       <c r="B222" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C222" s="2">
         <v>51130</v>
@@ -4269,12 +4265,12 @@
         <v>104</v>
       </c>
     </row>
-    <row r="223" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A223" s="2">
         <v>51</v>
       </c>
       <c r="B223" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C223" s="2">
         <v>51150</v>
@@ -4283,12 +4279,12 @@
         <v>105</v>
       </c>
     </row>
-    <row r="224" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A224" s="2">
         <v>51</v>
       </c>
       <c r="B224" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C224" s="2">
         <v>51170</v>
@@ -4297,12 +4293,12 @@
         <v>106</v>
       </c>
     </row>
-    <row r="225" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A225" s="2">
         <v>51</v>
       </c>
       <c r="B225" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C225" s="2">
         <v>51190</v>
@@ -4311,12 +4307,12 @@
         <v>107</v>
       </c>
     </row>
-    <row r="226" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A226" s="2">
         <v>51</v>
       </c>
       <c r="B226" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C226" s="2">
         <v>51210</v>
@@ -4325,12 +4321,12 @@
         <v>108</v>
       </c>
     </row>
-    <row r="227" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A227" s="2">
         <v>51</v>
       </c>
       <c r="B227" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C227" s="2">
         <v>51230</v>
@@ -4339,12 +4335,12 @@
         <v>109</v>
       </c>
     </row>
-    <row r="228" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A228" s="2">
         <v>51</v>
       </c>
       <c r="B228" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C228" s="2">
         <v>51720</v>
@@ -4353,12 +4349,12 @@
         <v>110</v>
       </c>
     </row>
-    <row r="229" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A229" s="2">
         <v>51</v>
       </c>
       <c r="B229" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C229" s="2">
         <v>51730</v>
@@ -4367,12 +4363,12 @@
         <v>111</v>
       </c>
     </row>
-    <row r="230" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A230" s="2">
         <v>51</v>
       </c>
       <c r="B230" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C230" s="2">
         <v>51750</v>
@@ -4381,12 +4377,12 @@
         <v>112</v>
       </c>
     </row>
-    <row r="231" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A231" s="2">
         <v>51</v>
       </c>
       <c r="B231" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C231" s="2">
         <v>51760</v>
@@ -4395,12 +4391,12 @@
         <v>113</v>
       </c>
     </row>
-    <row r="232" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A232" s="2">
         <v>51</v>
       </c>
       <c r="B232" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C232" s="2">
         <v>51770</v>
@@ -4409,12 +4405,12 @@
         <v>114</v>
       </c>
     </row>
-    <row r="233" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A233" s="2">
         <v>51</v>
       </c>
       <c r="B233" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C233" s="2">
         <v>51780</v>
@@ -4423,12 +4419,12 @@
         <v>115</v>
       </c>
     </row>
-    <row r="234" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A234" s="2">
         <v>51</v>
       </c>
       <c r="B234" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C234" s="2">
         <v>51790</v>
@@ -4437,12 +4433,12 @@
         <v>116</v>
       </c>
     </row>
-    <row r="235" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A235" s="2">
         <v>51</v>
       </c>
       <c r="B235" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C235" s="2">
         <v>51800</v>
@@ -4451,12 +4447,12 @@
         <v>117</v>
       </c>
     </row>
-    <row r="236" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A236" s="2">
         <v>51</v>
       </c>
       <c r="B236" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C236" s="2">
         <v>51810</v>
@@ -4465,12 +4461,12 @@
         <v>118</v>
       </c>
     </row>
-    <row r="237" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A237" s="2">
         <v>51</v>
       </c>
       <c r="B237" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C237" s="2">
         <v>51820</v>
@@ -4479,12 +4475,12 @@
         <v>119</v>
       </c>
     </row>
-    <row r="238" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A238" s="2">
         <v>51</v>
       </c>
       <c r="B238" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C238" s="2">
         <v>51830</v>
@@ -4493,12 +4489,12 @@
         <v>120</v>
       </c>
     </row>
-    <row r="239" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A239" s="2">
         <v>52</v>
       </c>
       <c r="B239" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C239" s="2">
         <v>52111</v>
@@ -4507,12 +4503,12 @@
         <v>153</v>
       </c>
     </row>
-    <row r="240" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A240" s="2">
         <v>52</v>
       </c>
       <c r="B240" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C240" s="2">
         <v>52113</v>
@@ -4521,12 +4517,12 @@
         <v>154</v>
       </c>
     </row>
-    <row r="241" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A241" s="2">
         <v>52</v>
       </c>
       <c r="B241" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C241" s="2">
         <v>52130</v>
@@ -4535,12 +4531,12 @@
         <v>155</v>
       </c>
     </row>
-    <row r="242" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A242" s="2">
         <v>52</v>
       </c>
       <c r="B242" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C242" s="2">
         <v>52140</v>
@@ -4549,12 +4545,12 @@
         <v>156</v>
       </c>
     </row>
-    <row r="243" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A243" s="2">
         <v>52</v>
       </c>
       <c r="B243" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C243" s="2">
         <v>52180</v>
@@ -4563,12 +4559,12 @@
         <v>157</v>
       </c>
     </row>
-    <row r="244" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A244" s="2">
         <v>52</v>
       </c>
       <c r="B244" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C244" s="2">
         <v>52190</v>
@@ -4577,12 +4573,12 @@
         <v>158</v>
       </c>
     </row>
-    <row r="245" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A245" s="2">
         <v>52</v>
       </c>
       <c r="B245" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C245" s="2">
         <v>52210</v>
@@ -4591,12 +4587,12 @@
         <v>159</v>
       </c>
     </row>
-    <row r="246" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A246" s="2">
         <v>52</v>
       </c>
       <c r="B246" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C246" s="2">
         <v>52710</v>
@@ -4605,12 +4601,12 @@
         <v>160</v>
       </c>
     </row>
-    <row r="247" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A247" s="2">
         <v>52</v>
       </c>
       <c r="B247" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C247" s="2">
         <v>52720</v>
@@ -4619,12 +4615,12 @@
         <v>161</v>
       </c>
     </row>
-    <row r="248" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A248" s="2">
         <v>52</v>
       </c>
       <c r="B248" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C248" s="2">
         <v>52730</v>
@@ -4633,12 +4629,12 @@
         <v>162</v>
       </c>
     </row>
-    <row r="249" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A249" s="2">
         <v>52</v>
       </c>
       <c r="B249" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C249" s="2">
         <v>52740</v>
@@ -4647,12 +4643,12 @@
         <v>163</v>
       </c>
     </row>
-    <row r="250" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A250" s="2">
         <v>52</v>
       </c>
       <c r="B250" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C250" s="2">
         <v>52750</v>
@@ -4661,12 +4657,12 @@
         <v>164</v>
       </c>
     </row>
-    <row r="251" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A251" s="2">
         <v>52</v>
       </c>
       <c r="B251" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C251" s="2">
         <v>52770</v>
@@ -4675,12 +4671,12 @@
         <v>165</v>
       </c>
     </row>
-    <row r="252" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A252" s="2">
         <v>52</v>
       </c>
       <c r="B252" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C252" s="2">
         <v>52790</v>
@@ -4689,12 +4685,12 @@
         <v>166</v>
       </c>
     </row>
-    <row r="253" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A253" s="2">
         <v>52</v>
       </c>
       <c r="B253" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C253" s="2">
         <v>52800</v>

</xml_diff>

<commit_message>
chore: remove temporary Excel file
</commit_message>
<xml_diff>
--- a/assets/region_codes.xlsx
+++ b/assets/region_codes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\SNOB\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C67998A-9111-49CF-81B8-236F02140736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11F756CF-04B4-48C9-A76B-0204BA2107ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -555,9 +555,6 @@
     <t>구례군</t>
   </si>
   <si>
-    <t>고흥군</t>
-  </si>
-  <si>
     <t>보성군</t>
   </si>
   <si>
@@ -779,6 +776,10 @@
   </si>
   <si>
     <t>전남광주통합특별시</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>고흥군</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1159,16 +1160,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>247</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.45">
@@ -1868,7 +1869,7 @@
         <v>27720</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.45">
@@ -2386,7 +2387,7 @@
         <v>41192</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.45">
@@ -2400,7 +2401,7 @@
         <v>41194</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.45">
@@ -2414,7 +2415,7 @@
         <v>41196</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.45">
@@ -3276,7 +3277,7 @@
         <v>46</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C152" s="2">
         <v>46110</v>
@@ -3290,7 +3291,7 @@
         <v>46</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C153" s="2">
         <v>46130</v>
@@ -3304,7 +3305,7 @@
         <v>46</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C154" s="2">
         <v>46150</v>
@@ -3318,7 +3319,7 @@
         <v>46</v>
       </c>
       <c r="B155" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C155" s="2">
         <v>46170</v>
@@ -3332,7 +3333,7 @@
         <v>46</v>
       </c>
       <c r="B156" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C156" s="2">
         <v>46230</v>
@@ -3346,7 +3347,7 @@
         <v>46</v>
       </c>
       <c r="B157" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C157" s="2">
         <v>46710</v>
@@ -3360,7 +3361,7 @@
         <v>46</v>
       </c>
       <c r="B158" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C158" s="2">
         <v>46720</v>
@@ -3374,7 +3375,7 @@
         <v>46</v>
       </c>
       <c r="B159" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C159" s="2">
         <v>46730</v>
@@ -3388,13 +3389,13 @@
         <v>46</v>
       </c>
       <c r="B160" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C160" s="2">
         <v>46770</v>
       </c>
       <c r="D160" s="3" t="s">
-        <v>176</v>
+        <v>249</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.45">
@@ -3402,13 +3403,13 @@
         <v>46</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C161" s="2">
         <v>46780</v>
       </c>
       <c r="D161" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.45">
@@ -3416,13 +3417,13 @@
         <v>46</v>
       </c>
       <c r="B162" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C162" s="2">
         <v>46790</v>
       </c>
       <c r="D162" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.45">
@@ -3430,13 +3431,13 @@
         <v>46</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C163" s="2">
         <v>46800</v>
       </c>
       <c r="D163" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.45">
@@ -3444,13 +3445,13 @@
         <v>46</v>
       </c>
       <c r="B164" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C164" s="2">
         <v>46810</v>
       </c>
       <c r="D164" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.45">
@@ -3458,13 +3459,13 @@
         <v>46</v>
       </c>
       <c r="B165" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C165" s="2">
         <v>46820</v>
       </c>
       <c r="D165" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.45">
@@ -3472,13 +3473,13 @@
         <v>46</v>
       </c>
       <c r="B166" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C166" s="2">
         <v>46830</v>
       </c>
       <c r="D166" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.45">
@@ -3486,13 +3487,13 @@
         <v>46</v>
       </c>
       <c r="B167" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C167" s="2">
         <v>46840</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.45">
@@ -3500,13 +3501,13 @@
         <v>46</v>
       </c>
       <c r="B168" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C168" s="2">
         <v>46860</v>
       </c>
       <c r="D168" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.45">
@@ -3514,13 +3515,13 @@
         <v>46</v>
       </c>
       <c r="B169" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C169" s="2">
         <v>46870</v>
       </c>
       <c r="D169" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.45">
@@ -3528,13 +3529,13 @@
         <v>46</v>
       </c>
       <c r="B170" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C170" s="2">
         <v>46880</v>
       </c>
       <c r="D170" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.45">
@@ -3542,13 +3543,13 @@
         <v>46</v>
       </c>
       <c r="B171" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C171" s="2">
         <v>46890</v>
       </c>
       <c r="D171" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.45">
@@ -3556,13 +3557,13 @@
         <v>46</v>
       </c>
       <c r="B172" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C172" s="2">
         <v>46900</v>
       </c>
       <c r="D172" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.45">
@@ -3570,13 +3571,13 @@
         <v>46</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C173" s="2">
         <v>46910</v>
       </c>
       <c r="D173" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.45">
@@ -3584,13 +3585,13 @@
         <v>47</v>
       </c>
       <c r="B174" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C174" s="2">
         <v>47111</v>
       </c>
       <c r="D174" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.45">
@@ -3598,13 +3599,13 @@
         <v>47</v>
       </c>
       <c r="B175" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C175" s="2">
         <v>47113</v>
       </c>
       <c r="D175" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.45">
@@ -3612,13 +3613,13 @@
         <v>47</v>
       </c>
       <c r="B176" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C176" s="2">
         <v>47130</v>
       </c>
       <c r="D176" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.45">
@@ -3626,13 +3627,13 @@
         <v>47</v>
       </c>
       <c r="B177" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C177" s="2">
         <v>47150</v>
       </c>
       <c r="D177" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.45">
@@ -3640,13 +3641,13 @@
         <v>47</v>
       </c>
       <c r="B178" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C178" s="2">
         <v>47170</v>
       </c>
       <c r="D178" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.45">
@@ -3654,13 +3655,13 @@
         <v>47</v>
       </c>
       <c r="B179" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C179" s="2">
         <v>47190</v>
       </c>
       <c r="D179" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.45">
@@ -3668,13 +3669,13 @@
         <v>47</v>
       </c>
       <c r="B180" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C180" s="2">
         <v>47210</v>
       </c>
       <c r="D180" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.45">
@@ -3682,13 +3683,13 @@
         <v>47</v>
       </c>
       <c r="B181" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C181" s="2">
         <v>47230</v>
       </c>
       <c r="D181" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.45">
@@ -3696,13 +3697,13 @@
         <v>47</v>
       </c>
       <c r="B182" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C182" s="2">
         <v>47250</v>
       </c>
       <c r="D182" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.45">
@@ -3710,13 +3711,13 @@
         <v>47</v>
       </c>
       <c r="B183" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C183" s="2">
         <v>47280</v>
       </c>
       <c r="D183" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.45">
@@ -3724,13 +3725,13 @@
         <v>47</v>
       </c>
       <c r="B184" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C184" s="2">
         <v>47290</v>
       </c>
       <c r="D184" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.45">
@@ -3738,13 +3739,13 @@
         <v>47</v>
       </c>
       <c r="B185" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C185" s="2">
         <v>47730</v>
       </c>
       <c r="D185" s="3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.45">
@@ -3752,13 +3753,13 @@
         <v>47</v>
       </c>
       <c r="B186" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C186" s="2">
         <v>47750</v>
       </c>
       <c r="D186" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.45">
@@ -3766,13 +3767,13 @@
         <v>47</v>
       </c>
       <c r="B187" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C187" s="2">
         <v>47760</v>
       </c>
       <c r="D187" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.45">
@@ -3780,13 +3781,13 @@
         <v>47</v>
       </c>
       <c r="B188" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C188" s="2">
         <v>47770</v>
       </c>
       <c r="D188" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.45">
@@ -3794,13 +3795,13 @@
         <v>47</v>
       </c>
       <c r="B189" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C189" s="2">
         <v>47820</v>
       </c>
       <c r="D189" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.45">
@@ -3808,13 +3809,13 @@
         <v>47</v>
       </c>
       <c r="B190" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C190" s="2">
         <v>47830</v>
       </c>
       <c r="D190" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.45">
@@ -3822,13 +3823,13 @@
         <v>47</v>
       </c>
       <c r="B191" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C191" s="2">
         <v>47840</v>
       </c>
       <c r="D191" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.45">
@@ -3836,13 +3837,13 @@
         <v>47</v>
       </c>
       <c r="B192" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C192" s="2">
         <v>47850</v>
       </c>
       <c r="D192" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.45">
@@ -3850,13 +3851,13 @@
         <v>47</v>
       </c>
       <c r="B193" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C193" s="2">
         <v>47900</v>
       </c>
       <c r="D193" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.45">
@@ -3864,13 +3865,13 @@
         <v>47</v>
       </c>
       <c r="B194" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C194" s="2">
         <v>47920</v>
       </c>
       <c r="D194" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.45">
@@ -3878,13 +3879,13 @@
         <v>47</v>
       </c>
       <c r="B195" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C195" s="2">
         <v>47930</v>
       </c>
       <c r="D195" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.45">
@@ -3892,13 +3893,13 @@
         <v>47</v>
       </c>
       <c r="B196" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C196" s="2">
         <v>47940</v>
       </c>
       <c r="D196" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.45">
@@ -3906,13 +3907,13 @@
         <v>48</v>
       </c>
       <c r="B197" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C197" s="2">
         <v>48121</v>
       </c>
       <c r="D197" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.45">
@@ -3920,13 +3921,13 @@
         <v>48</v>
       </c>
       <c r="B198" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C198" s="2">
         <v>48123</v>
       </c>
       <c r="D198" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.45">
@@ -3934,13 +3935,13 @@
         <v>48</v>
       </c>
       <c r="B199" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C199" s="2">
         <v>48125</v>
       </c>
       <c r="D199" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.45">
@@ -3948,13 +3949,13 @@
         <v>48</v>
       </c>
       <c r="B200" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C200" s="2">
         <v>48127</v>
       </c>
       <c r="D200" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.45">
@@ -3962,13 +3963,13 @@
         <v>48</v>
       </c>
       <c r="B201" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C201" s="2">
         <v>48129</v>
       </c>
       <c r="D201" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.45">
@@ -3976,13 +3977,13 @@
         <v>48</v>
       </c>
       <c r="B202" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C202" s="2">
         <v>48170</v>
       </c>
       <c r="D202" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.45">
@@ -3990,13 +3991,13 @@
         <v>48</v>
       </c>
       <c r="B203" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C203" s="2">
         <v>48220</v>
       </c>
       <c r="D203" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.45">
@@ -4004,13 +4005,13 @@
         <v>48</v>
       </c>
       <c r="B204" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C204" s="2">
         <v>48240</v>
       </c>
       <c r="D204" s="3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.45">
@@ -4018,13 +4019,13 @@
         <v>48</v>
       </c>
       <c r="B205" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C205" s="2">
         <v>48250</v>
       </c>
       <c r="D205" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.45">
@@ -4032,13 +4033,13 @@
         <v>48</v>
       </c>
       <c r="B206" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C206" s="2">
         <v>48270</v>
       </c>
       <c r="D206" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.45">
@@ -4046,13 +4047,13 @@
         <v>48</v>
       </c>
       <c r="B207" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C207" s="2">
         <v>48310</v>
       </c>
       <c r="D207" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.45">
@@ -4060,13 +4061,13 @@
         <v>48</v>
       </c>
       <c r="B208" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C208" s="2">
         <v>48330</v>
       </c>
       <c r="D208" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.45">
@@ -4074,13 +4075,13 @@
         <v>48</v>
       </c>
       <c r="B209" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C209" s="2">
         <v>48720</v>
       </c>
       <c r="D209" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.45">
@@ -4088,13 +4089,13 @@
         <v>48</v>
       </c>
       <c r="B210" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C210" s="2">
         <v>48730</v>
       </c>
       <c r="D210" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.45">
@@ -4102,13 +4103,13 @@
         <v>48</v>
       </c>
       <c r="B211" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C211" s="2">
         <v>48740</v>
       </c>
       <c r="D211" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.45">
@@ -4116,7 +4117,7 @@
         <v>48</v>
       </c>
       <c r="B212" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C212" s="2">
         <v>48820</v>
@@ -4130,13 +4131,13 @@
         <v>48</v>
       </c>
       <c r="B213" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C213" s="2">
         <v>48840</v>
       </c>
       <c r="D213" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.45">
@@ -4144,13 +4145,13 @@
         <v>48</v>
       </c>
       <c r="B214" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C214" s="2">
         <v>48850</v>
       </c>
       <c r="D214" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.45">
@@ -4158,13 +4159,13 @@
         <v>48</v>
       </c>
       <c r="B215" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C215" s="2">
         <v>48860</v>
       </c>
       <c r="D215" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.45">
@@ -4172,13 +4173,13 @@
         <v>48</v>
       </c>
       <c r="B216" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C216" s="2">
         <v>48870</v>
       </c>
       <c r="D216" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.45">
@@ -4186,13 +4187,13 @@
         <v>48</v>
       </c>
       <c r="B217" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C217" s="2">
         <v>48880</v>
       </c>
       <c r="D217" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.45">
@@ -4200,13 +4201,13 @@
         <v>48</v>
       </c>
       <c r="B218" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C218" s="2">
         <v>48890</v>
       </c>
       <c r="D218" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.45">
@@ -4214,13 +4215,13 @@
         <v>50</v>
       </c>
       <c r="B219" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C219" s="2">
         <v>50110</v>
       </c>
       <c r="D219" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.45">
@@ -4228,13 +4229,13 @@
         <v>50</v>
       </c>
       <c r="B220" s="3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C220" s="2">
         <v>50130</v>
       </c>
       <c r="D220" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.45">
@@ -4242,7 +4243,7 @@
         <v>51</v>
       </c>
       <c r="B221" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C221" s="2">
         <v>51110</v>
@@ -4256,7 +4257,7 @@
         <v>51</v>
       </c>
       <c r="B222" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C222" s="2">
         <v>51130</v>
@@ -4270,7 +4271,7 @@
         <v>51</v>
       </c>
       <c r="B223" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C223" s="2">
         <v>51150</v>
@@ -4284,7 +4285,7 @@
         <v>51</v>
       </c>
       <c r="B224" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C224" s="2">
         <v>51170</v>
@@ -4298,7 +4299,7 @@
         <v>51</v>
       </c>
       <c r="B225" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C225" s="2">
         <v>51190</v>
@@ -4312,7 +4313,7 @@
         <v>51</v>
       </c>
       <c r="B226" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C226" s="2">
         <v>51210</v>
@@ -4326,7 +4327,7 @@
         <v>51</v>
       </c>
       <c r="B227" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C227" s="2">
         <v>51230</v>
@@ -4340,7 +4341,7 @@
         <v>51</v>
       </c>
       <c r="B228" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C228" s="2">
         <v>51720</v>
@@ -4354,7 +4355,7 @@
         <v>51</v>
       </c>
       <c r="B229" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C229" s="2">
         <v>51730</v>
@@ -4368,7 +4369,7 @@
         <v>51</v>
       </c>
       <c r="B230" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C230" s="2">
         <v>51750</v>
@@ -4382,7 +4383,7 @@
         <v>51</v>
       </c>
       <c r="B231" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C231" s="2">
         <v>51760</v>
@@ -4396,7 +4397,7 @@
         <v>51</v>
       </c>
       <c r="B232" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C232" s="2">
         <v>51770</v>
@@ -4410,7 +4411,7 @@
         <v>51</v>
       </c>
       <c r="B233" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C233" s="2">
         <v>51780</v>
@@ -4424,7 +4425,7 @@
         <v>51</v>
       </c>
       <c r="B234" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C234" s="2">
         <v>51790</v>
@@ -4438,7 +4439,7 @@
         <v>51</v>
       </c>
       <c r="B235" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C235" s="2">
         <v>51800</v>
@@ -4452,7 +4453,7 @@
         <v>51</v>
       </c>
       <c r="B236" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C236" s="2">
         <v>51810</v>
@@ -4466,7 +4467,7 @@
         <v>51</v>
       </c>
       <c r="B237" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C237" s="2">
         <v>51820</v>
@@ -4480,7 +4481,7 @@
         <v>51</v>
       </c>
       <c r="B238" s="3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C238" s="2">
         <v>51830</v>
@@ -4494,7 +4495,7 @@
         <v>52</v>
       </c>
       <c r="B239" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C239" s="2">
         <v>52111</v>
@@ -4508,7 +4509,7 @@
         <v>52</v>
       </c>
       <c r="B240" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C240" s="2">
         <v>52113</v>
@@ -4522,7 +4523,7 @@
         <v>52</v>
       </c>
       <c r="B241" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C241" s="2">
         <v>52130</v>
@@ -4536,7 +4537,7 @@
         <v>52</v>
       </c>
       <c r="B242" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C242" s="2">
         <v>52140</v>
@@ -4550,7 +4551,7 @@
         <v>52</v>
       </c>
       <c r="B243" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C243" s="2">
         <v>52180</v>
@@ -4564,7 +4565,7 @@
         <v>52</v>
       </c>
       <c r="B244" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C244" s="2">
         <v>52190</v>
@@ -4578,7 +4579,7 @@
         <v>52</v>
       </c>
       <c r="B245" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C245" s="2">
         <v>52210</v>
@@ -4592,7 +4593,7 @@
         <v>52</v>
       </c>
       <c r="B246" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C246" s="2">
         <v>52710</v>
@@ -4606,7 +4607,7 @@
         <v>52</v>
       </c>
       <c r="B247" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C247" s="2">
         <v>52720</v>
@@ -4620,7 +4621,7 @@
         <v>52</v>
       </c>
       <c r="B248" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C248" s="2">
         <v>52730</v>
@@ -4634,7 +4635,7 @@
         <v>52</v>
       </c>
       <c r="B249" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C249" s="2">
         <v>52740</v>
@@ -4648,7 +4649,7 @@
         <v>52</v>
       </c>
       <c r="B250" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C250" s="2">
         <v>52750</v>
@@ -4662,7 +4663,7 @@
         <v>52</v>
       </c>
       <c r="B251" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C251" s="2">
         <v>52770</v>
@@ -4676,7 +4677,7 @@
         <v>52</v>
       </c>
       <c r="B252" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C252" s="2">
         <v>52790</v>
@@ -4690,7 +4691,7 @@
         <v>52</v>
       </c>
       <c r="B253" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C253" s="2">
         <v>52800</v>

</xml_diff>